<commit_message>
improved config from excel table, added return all tables on a sheet as json object
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/testconfigfromexceltablegetattributeasi32.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/testconfigfromexceltablegetattributeasi32.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4034be38423d4008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R25f795e2210b40dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
@@ -67,7 +67,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3901a9e3c24d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51152020b21e47aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>